<commit_message>
Regenerated the plots and tables again with new results.
</commit_message>
<xml_diff>
--- a/analysis/06-if/tables/if_gemma4_latest.xlsx
+++ b/analysis/06-if/tables/if_gemma4_latest.xlsx
@@ -357,32 +357,32 @@
     <row r="1" s="1" customFormat="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Verse</t>
+          <t>verse</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Line</t>
+          <t>line</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Text</t>
+          <t>text</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Sentiment</t>
+          <t>gemma4_sentiment</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>confidence_score</t>
+          <t>gemma4_conf</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>reasoning</t>
+          <t>gemma4_reasoning</t>
         </is>
       </c>
     </row>
@@ -400,15 +400,15 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Anticipation</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="E2">
-        <v>0.75</v>
+        <v>0.8</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>The phrase is incomplete and suggests a test or challenge that is yet to come.</t>
+          <t>The phrase is an incomplete, proverbial statement that lacks strong emotional content.</t>
         </is>
       </c>
     </row>
@@ -430,11 +430,11 @@
         </is>
       </c>
       <c r="E3">
-        <v>0.95</v>
+        <v>0.9</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>The phrase implies betrayal and accusation ('losing theirs and blaming it on you')</t>
+          <t>The phrase describes an act of betrayal and false accusation, which evokes strong feelings of injustice and anger.</t>
         </is>
       </c>
     </row>
@@ -456,11 +456,11 @@
         </is>
       </c>
       <c r="E4">
-        <v>0.95</v>
+        <v>0.9</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>The text explicitly discusses the concept of self-trust amidst external doubt.</t>
+          <t>The phrase directly addresses the concept of self-reliance and belief in one's own character.</t>
         </is>
       </c>
     </row>
@@ -478,15 +478,15 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Anticipation</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="E5">
-        <v>0.65</v>
+        <v>0.6</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>The phrase suggests a need to prepare for or consider future doubts/uncertainties.</t>
+          <t>The phrase is a directive or suggestion that lacks strong emotional coloring.</t>
         </is>
       </c>
     </row>
@@ -504,15 +504,15 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Anticipation</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="E6">
-        <v>0.75</v>
+        <v>0.6</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>The conditional nature ('if you can wait') suggests a hopeful or expectant state regarding a future event</t>
+          <t>The phrase is a conditional statement that lacks strong emotional markers.</t>
         </is>
       </c>
     </row>
@@ -530,15 +530,15 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Anger</t>
+          <t>Disgust</t>
         </is>
       </c>
       <c r="E7">
-        <v>0.95</v>
+        <v>0.9</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Direct prohibition against dishonesty and betrayal</t>
+          <t>The phrase 'being lied about' and the command 'don't deal in lies' convey strong moral revulsion.</t>
         </is>
       </c>
     </row>
@@ -560,11 +560,11 @@
         </is>
       </c>
       <c r="E8">
-        <v>0.65</v>
+        <v>0.6</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>The text is a philosophical caution or piece of advice that lacks strong emotional markers.</t>
+          <t>The text is a philosophical caution rather than an expression of strong emotion.</t>
         </is>
       </c>
     </row>
@@ -586,11 +586,11 @@
         </is>
       </c>
       <c r="E9">
-        <v>0.65</v>
+        <v>0.6</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>A cautionary or advisory tone that is more observational than emotionally charged</t>
+          <t>The phrase is a piece of advice or caution that lacks strong emotional coloring.</t>
         </is>
       </c>
     </row>
@@ -608,15 +608,15 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Anticipation</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="E10">
-        <v>0.75</v>
+        <v>0.8</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>The conditional 'if' and the advice structure suggest a hopeful possibility or future state.</t>
+          <t>The text is philosophical and advisory, lacking strong emotional markers.</t>
         </is>
       </c>
     </row>
@@ -638,11 +638,11 @@
         </is>
       </c>
       <c r="E11">
-        <v>0.65</v>
+        <v>0.8</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Philosophical instruction that is objective and instructional in tone</t>
+          <t>The text is a philosophical instruction that lacks strong emotional markers.</t>
         </is>
       </c>
     </row>
@@ -660,15 +660,15 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Anticipation</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="E12">
-        <v>0.75</v>
+        <v>0.6</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>The phrasing suggests a contemplation or expectation of encountering extreme opposing forces.</t>
+          <t>The phrase is a rhetorical question that presents opposing concepts without emotional context.</t>
         </is>
       </c>
     </row>
@@ -690,11 +690,11 @@
         </is>
       </c>
       <c r="E13">
-        <v>0.75</v>
+        <v>0.8</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>The imperative tone and use of 'impostors' suggest strong disapproval or rage.</t>
+          <t>The imperative tone and the derogatory term 'impostors' suggest strong displeasure or rage.</t>
         </is>
       </c>
     </row>
@@ -712,15 +712,15 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Fear</t>
+          <t>Sadness</t>
         </is>
       </c>
       <c r="E14">
-        <v>0.9</v>
+        <v>0.8</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>The phrase implies dread or apprehension regarding a difficult revelation.</t>
+          <t>The phrasing suggests a difficult, painful truth that the speaker fears the listener cannot handle.</t>
         </is>
       </c>
     </row>
@@ -742,11 +742,11 @@
         </is>
       </c>
       <c r="E15">
-        <v>0.95</v>
+        <v>0.9</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>The phrase 'twisted by knaves' suggests betrayal and malicious intent.</t>
+          <t>The language suggests betrayal and malicious intent, which evokes anger.</t>
         </is>
       </c>
     </row>
@@ -768,11 +768,11 @@
         </is>
       </c>
       <c r="E16">
-        <v>0.95</v>
+        <v>0.9</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>The phrase 'broken' applied to deeply invested things suggests loss and disappointment.</t>
+          <t>The phrase 'broken' applied to things given one's life suggests loss and deep disappointment.</t>
         </is>
       </c>
     </row>
@@ -794,11 +794,11 @@
         </is>
       </c>
       <c r="E17">
-        <v>0.65</v>
+        <v>0.8</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>The phrase is descriptive and action-oriented without clear emotional context.</t>
+          <t>The text is a descriptive, action-oriented phrase lacking strong emotional indicators.</t>
         </is>
       </c>
     </row>
@@ -816,15 +816,15 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Anticipation</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="E18">
-        <v>0.75</v>
+        <v>0.8</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>The phrase suggests a future goal or reward that is being looked forward to.</t>
+          <t>The text is a fragment of a song lyric that lacks strong emotional context on its own.</t>
         </is>
       </c>
     </row>
@@ -850,7 +850,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>The phrase suggests a moment of high stakes and waiting for an outcome.</t>
+          <t>The phrase suggests a moment of decision and waiting for a potential outcome.</t>
         </is>
       </c>
     </row>
@@ -872,11 +872,11 @@
         </is>
       </c>
       <c r="E20">
-        <v>0.75</v>
+        <v>0.8</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>The phrase 'lose' suggests loss or failure, leading to a melancholic sense of starting over.</t>
+          <t>The phrase suggests a cycle of loss and forced restarts, implying melancholy or resignation.</t>
         </is>
       </c>
     </row>
@@ -894,15 +894,15 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Anger</t>
+          <t>Fear</t>
         </is>
       </c>
       <c r="E21">
-        <v>0.95</v>
+        <v>0.8</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>The imperative command 'never breathe' suggests prohibition and forceful displeasure.</t>
+          <t>The command suggests a need for secrecy and suppression, implying a fear of negative consequences if the truth is revealed.</t>
         </is>
       </c>
     </row>
@@ -920,15 +920,15 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Anticipation</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="E22">
-        <v>0.75</v>
+        <v>0.8</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>The phrase suggests a build-up of effort or potential action.</t>
+          <t>The phrase is a fragment of a rhetorical or descriptive passage lacking clear emotional context.</t>
         </is>
       </c>
     </row>
@@ -954,7 +954,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>The phrase 'long after they are gone' suggests loss and enduring grief.</t>
+          <t>The phrase suggests a lingering, painful duty or memory of something lost.</t>
         </is>
       </c>
     </row>
@@ -976,11 +976,11 @@
         </is>
       </c>
       <c r="E24">
-        <v>0.9</v>
+        <v>0.8</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>The phrase suggests emptiness or lack of emotional substance.</t>
+          <t>The phrase suggests a state of emptiness or emotional depletion, which aligns with sadness.</t>
         </is>
       </c>
     </row>
@@ -1002,11 +1002,11 @@
         </is>
       </c>
       <c r="E25">
-        <v>0.75</v>
+        <v>0.8</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>The exclamation 'Hold on!' creates a sense of pause and expectation for what follows.</t>
+          <t>The phrase 'Hold on!' suggests a pause and a wait for something to come next.</t>
         </is>
       </c>
     </row>
@@ -1024,15 +1024,15 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Anticipation</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="E26">
-        <v>0.75</v>
+        <v>0.8</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>The phrasing suggests a challenge or promise of future capability/success.</t>
+          <t>The text is a piece of advice or a maxim, presenting a balanced, objective statement.</t>
         </is>
       </c>
     </row>
@@ -1050,15 +1050,15 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Anticipation</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="E27">
-        <v>0.65</v>
+        <v>0.8</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>The phrase suggests a choice or path forward that requires careful consideration and potential future action.</t>
+          <t>The phrase is a piece of advice or a statement of balance, lacking strong emotional markers.</t>
         </is>
       </c>
     </row>
@@ -1076,15 +1076,15 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Anticipation</t>
+          <t>Joy</t>
         </is>
       </c>
       <c r="E28">
-        <v>0.75</v>
+        <v>0.8</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>The conditional structure suggests a future state or realization of safety/freedom from pain.</t>
+          <t>The statement suggests a state of emotional invulnerability and safety, which evokes a feeling of happiness.</t>
         </is>
       </c>
     </row>
@@ -1102,15 +1102,15 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Sadness</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="E29">
-        <v>0.75</v>
+        <v>0.8</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>The phrase suggests a feeling of being valued moderately ('count') but not deeply or fully appreciated ('none too much').</t>
+          <t>The phrase is a balanced, reflective statement that lacks strong emotional markers.</t>
         </is>
       </c>
     </row>
@@ -1128,15 +1128,15 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Anticipation</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="E30">
-        <v>0.75</v>
+        <v>0.8</v>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>The phrase suggests waiting for or needing to complete a difficult passage of time.</t>
+          <t>The phrase is incomplete and highly abstract, making a definitive emotional judgment difficult.</t>
         </is>
       </c>
     </row>
@@ -1158,11 +1158,11 @@
         </is>
       </c>
       <c r="E31">
-        <v>0.65</v>
+        <v>0.9</v>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>The phrase is purely descriptive and lacks explicit emotional content.</t>
+          <t>The text is a simple, factual statement of distance covered without emotional context.</t>
         </is>
       </c>
     </row>
@@ -1180,15 +1180,15 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Joy</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="E32">
-        <v>0.75</v>
+        <v>0.8</v>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>A declaration of ownership or possession over something vast and valuable</t>
+          <t>The statement is a declarative claim of ownership without strong emotional indicators.</t>
         </is>
       </c>
     </row>
@@ -1210,11 +1210,11 @@
         </is>
       </c>
       <c r="E33">
-        <v>0.95</v>
+        <v>0.9</v>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Exclamatory declaration of positive life event and pride</t>
+          <t>The exclamation and declaration of a significant life event suggest overwhelming happiness and pride.</t>
         </is>
       </c>
     </row>

</xml_diff>